<commit_message>
Data stored in excel file for local and security.
</commit_message>
<xml_diff>
--- a/chat_data.xlsx
+++ b/chat_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,7 +963,49 @@
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-27 19:46:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-27 19:46:10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>cls</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>